<commit_message>
Update Light Proximity Switch BOM components and pricing
Revised the Bill of Materials for the Light Proximity Switch to update suppliers, manufacturers, part numbers, and pricing. Notable changes include switching the op-amp to MCP6231-E/P, updating several component sources to DigiKey and Amazon, and adjusting unit/build costs. The Excel BOM was also updated to reflect these changes.
</commit_message>
<xml_diff>
--- a/Documentation/Working Docs/Light_Proximity_Switch_BOM.xlsx
+++ b/Documentation/Working Docs/Light_Proximity_Switch_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://neilsquiresoc.sharepoint.com/sites/Jake/Shared Documents/General/GitHub/Light-Proximity-Switch/Documentation/Working Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{F492F737-9929-49A8-B75C-5CA0CFD0A818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC45452C-4675-42C1-87B9-0F1C9DF2ACE9}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="13_ncr:1_{F492F737-9929-49A8-B75C-5CA0CFD0A818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A48A42F5-DC9E-47DD-8BFC-C6325B47EDF3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electronics" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="153">
   <si>
     <t>Qty</t>
   </si>
@@ -66,21 +66,6 @@
     <t>IC1</t>
   </si>
   <si>
-    <t>IC Op amp Single</t>
-  </si>
-  <si>
-    <t>Texas Instruments</t>
-  </si>
-  <si>
-    <t>TLV2451</t>
-  </si>
-  <si>
-    <t xml:space="preserve">296-1889-5-ND </t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/products/en?keywords=296-1889-5-ND%20</t>
-  </si>
-  <si>
     <t>Q1,Q2</t>
   </si>
   <si>
@@ -93,12 +78,6 @@
     <t>IRLD110PBF</t>
   </si>
   <si>
-    <t>IRLD110PBF-ND</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/product-detail/en/vishay-siliconix/IRLD110PBF/IRLD110PBF-ND/812489</t>
-  </si>
-  <si>
     <t>D1,D3</t>
   </si>
   <si>
@@ -123,36 +102,12 @@
     <t>Schottky diode 1N5817</t>
   </si>
   <si>
-    <t>Micro Commercial Co</t>
-  </si>
-  <si>
-    <t>1N5908</t>
-  </si>
-  <si>
-    <t>1N5817-TPCT-ND</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/products/en?keywords=1N5817-TPCT-ND</t>
-  </si>
-  <si>
     <t>LED1</t>
   </si>
   <si>
     <t xml:space="preserve">	LED GREEN CLEAR 5MM ROUND</t>
   </si>
   <si>
-    <t>Cree</t>
-  </si>
-  <si>
-    <t>C566C-GFF-CX0Y0892</t>
-  </si>
-  <si>
-    <t>C566C-GFF-CX0Y0892CT-ND</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/product-detail/en/cree-inc/C566C-GFF-CX0Y0892/C566C-GFF-CX0Y0892CT-ND/6138564</t>
-  </si>
-  <si>
     <t>C1</t>
   </si>
   <si>
@@ -210,12 +165,6 @@
     <t>C315C105K3R5TA</t>
   </si>
   <si>
-    <t xml:space="preserve">399-9714-ND	</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/product-detail/en/kemet/C315C105K3R5TA/399-9714-ND</t>
-  </si>
-  <si>
     <t>R1</t>
   </si>
   <si>
@@ -336,21 +285,9 @@
     <t>https://www.amazon.ca/AmazonBasics-Lithium-CR2032-Batteries-10-Pack/dp/B07RXJ4S7Z</t>
   </si>
   <si>
-    <t>Zip Tie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable Ties NYLON 2.8 12LBS </t>
-  </si>
-  <si>
     <t xml:space="preserve">Panduit </t>
   </si>
   <si>
-    <t xml:space="preserve">PLT.6SM-M </t>
-  </si>
-  <si>
-    <t>https://www.mouser.ca/ProductDetail/Panduit/PLT6SM-M?qs=kmt7eZ%252BGAiGfTZhDsQ7DXg%3D%3D</t>
-  </si>
-  <si>
     <t>Screws</t>
   </si>
   <si>
@@ -363,9 +300,6 @@
     <t>RM2X8MM 2701</t>
   </si>
   <si>
-    <t>335-155-ND</t>
-  </si>
-  <si>
     <t>https://www.digikey.ca/product-detail/en/apm-hexseal/RM2X8MM-2701/335-1155-ND/612919</t>
   </si>
   <si>
@@ -484,6 +418,81 @@
   </si>
   <si>
     <t>$1 per square inch, 100 square inch minimum.</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/stmicroelectronics/1N5817/770963</t>
+  </si>
+  <si>
+    <t>STMicroelectronics</t>
+  </si>
+  <si>
+    <t>1N5817</t>
+  </si>
+  <si>
+    <t>497-4547-1-ND</t>
+  </si>
+  <si>
+    <t>Cree LED</t>
+  </si>
+  <si>
+    <t>C566D-GFF-CY14Q7S1</t>
+  </si>
+  <si>
+    <t>C566D-GFF-CY14Q7S1-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/cree-led/C566D-GFF-CY14Q7S1/4793750</t>
+  </si>
+  <si>
+    <t>399-9714-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/kemet/C315C105K3R5TA/3726118</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>DigiKey</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Cable Tie</t>
+  </si>
+  <si>
+    <t>335-1155-ND</t>
+  </si>
+  <si>
+    <t>IC OPAMP GP 1 CIRCUIT 8DIP</t>
+  </si>
+  <si>
+    <t>Microchip Technology</t>
+  </si>
+  <si>
+    <t>MCP6231-E/P</t>
+  </si>
+  <si>
+    <t>MCP6231-E/P-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/microchip-technology/MCP6231-E-P/716239?s=N4IgTCBcDaILIGEAKA2MBmAjAWgKIHolsA5AERAF0BfIA</t>
+  </si>
+  <si>
+    <t>Cable Tie, Nylon, 71 mm long, 1.8 mm wide</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/panduit-corp/PLT-6SM-C/280029</t>
+  </si>
+  <si>
+    <t>PLT.6SM-C</t>
+  </si>
+  <si>
+    <t>https://www.amazon.ca/10PCS-IRLD110-DIP4-IRLD110PBF-DIP-4/dp/B0DSSJTPH8</t>
   </si>
 </sst>
 </file>
@@ -495,7 +504,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -525,12 +534,6 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0563C1"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -596,34 +599,33 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -711,6 +713,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1010,50 +1016,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:L20"/>
+  <dimension ref="B1:M20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="8.5703125" customWidth="1"/>
+    <col min="2" max="2" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" customWidth="1"/>
     <col min="4" max="4" width="37.140625" customWidth="1"/>
-    <col min="5" max="5" width="35.85546875" customWidth="1"/>
-    <col min="6" max="6" width="20.5703125" customWidth="1"/>
-    <col min="7" max="7" width="23.42578125" customWidth="1"/>
-    <col min="8" max="9" width="17.5703125" customWidth="1"/>
-    <col min="10" max="10" width="303.5703125" customWidth="1"/>
-    <col min="11" max="1028" width="8.5703125" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="303.5703125" customWidth="1"/>
+    <col min="12" max="1029" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B1" s="13" t="s">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="I1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>1</v>
       </c>
@@ -1061,568 +1072,615 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>143</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>139</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>144</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="10">
-        <v>2.89</v>
-      </c>
-      <c r="I2" s="10">
-        <f>H2*B2</f>
-        <v>2.89</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="H2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I2" s="9">
+        <v>0.69</v>
+      </c>
+      <c r="J2" s="9">
+        <f>I2*B2</f>
+        <v>0.69</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" s="9">
+        <v>1.63</v>
+      </c>
+      <c r="J3" s="9">
+        <f t="shared" ref="J3:J13" si="0">I3*B3</f>
+        <v>3.26</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="10">
-        <v>1.32</v>
-      </c>
-      <c r="I3" s="10">
-        <f t="shared" ref="I3:I14" si="0">H3*B3</f>
-        <v>2.64</v>
-      </c>
-      <c r="J3" s="2" t="s">
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" t="s">
-        <v>22</v>
-      </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>139</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" s="10">
-        <v>1.47</v>
+        <v>129</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>131</v>
       </c>
       <c r="I4" s="10">
-        <f t="shared" si="0"/>
-        <v>2.94</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+        <v>0.33</v>
+      </c>
+      <c r="J4" s="9">
+        <f t="shared" si="0"/>
+        <v>0.33</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>28</v>
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="11">
-        <v>0.26</v>
-      </c>
-      <c r="I5" s="10">
-        <f t="shared" si="0"/>
-        <v>0.26</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="F5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5" t="s">
+        <v>133</v>
+      </c>
+      <c r="H5" t="s">
+        <v>134</v>
+      </c>
+      <c r="I5" s="9">
+        <v>0.43</v>
+      </c>
+      <c r="J5" s="9">
+        <f t="shared" si="0"/>
+        <v>0.43</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" t="s">
+        <v>139</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="J6" s="9">
+        <f t="shared" si="0"/>
+        <v>0.4</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D6" t="s">
+      <c r="I7" s="9">
+        <v>0.54</v>
+      </c>
+      <c r="J7" s="9">
+        <f t="shared" si="0"/>
+        <v>1.08</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E6" t="s">
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>35</v>
       </c>
-      <c r="F6" t="s">
+      <c r="D8" t="s">
         <v>36</v>
       </c>
-      <c r="G6" t="s">
+      <c r="E8" t="s">
+        <v>139</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="10">
-        <v>0.33</v>
-      </c>
-      <c r="I6" s="10">
-        <f t="shared" si="0"/>
-        <v>0.33</v>
-      </c>
-      <c r="J6" s="2" t="s">
+      <c r="H8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="I8" s="9">
+        <v>0.35</v>
+      </c>
+      <c r="J8" s="9">
+        <f t="shared" si="0"/>
+        <v>0.35</v>
+      </c>
+      <c r="K8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="10">
-        <v>0.37</v>
-      </c>
-      <c r="I7" s="10">
-        <f t="shared" si="0"/>
-        <v>0.37</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="10">
-        <v>0.47</v>
-      </c>
-      <c r="I8" s="10">
-        <f t="shared" si="0"/>
-        <v>0.94</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>139</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" s="10">
-        <v>0.37</v>
-      </c>
-      <c r="I9" s="10">
-        <f t="shared" si="0"/>
-        <v>0.37</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="H9" t="s">
+        <v>136</v>
+      </c>
+      <c r="I9" s="9">
+        <v>1.32</v>
+      </c>
+      <c r="J9" s="9">
+        <f t="shared" si="0"/>
+        <v>1.32</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>139</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
-      </c>
-      <c r="H10" s="10">
-        <v>1.1299999999999999</v>
-      </c>
-      <c r="I10" s="10">
-        <f t="shared" si="0"/>
-        <v>1.1299999999999999</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="I10" s="9">
+        <v>3.39</v>
+      </c>
+      <c r="J10" s="9">
+        <f t="shared" si="0"/>
+        <v>3.39</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" t="s">
-        <v>61</v>
+      <c r="C11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="H11" s="10">
-        <v>3.79</v>
-      </c>
-      <c r="I11" s="10">
-        <f t="shared" si="0"/>
-        <v>3.79</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="I11" s="9">
+        <v>0.15</v>
+      </c>
+      <c r="J11" s="9">
+        <f t="shared" si="0"/>
+        <v>0.15</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>1</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" t="s">
+        <v>139</v>
+      </c>
+      <c r="F12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" t="s">
+        <v>57</v>
+      </c>
+      <c r="H12" t="s">
+        <v>58</v>
+      </c>
+      <c r="I12" s="9">
+        <v>0.15</v>
+      </c>
+      <c r="J12" s="9">
+        <f t="shared" si="0"/>
+        <v>0.15</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="7">
+        <v>1</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" t="s">
+        <v>139</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I13" s="11">
+        <v>1.88</v>
+      </c>
+      <c r="J13" s="9">
+        <f t="shared" si="0"/>
+        <v>1.88</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
         <v>66</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D14" t="s">
         <v>67</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E14" t="s">
+        <v>139</v>
+      </c>
+      <c r="F14" t="s">
         <v>68</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="G14" t="s">
         <v>69</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="H14" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="10">
-        <v>0.15</v>
-      </c>
-      <c r="I12" s="10">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
-      </c>
-      <c r="J12" s="3" t="s">
+      <c r="I14" s="9">
+        <v>1.21</v>
+      </c>
+      <c r="J14" s="9">
+        <f>I14*B14</f>
+        <v>1.21</v>
+      </c>
+      <c r="K14" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" t="s">
-        <v>68</v>
-      </c>
-      <c r="F13" t="s">
-        <v>74</v>
-      </c>
-      <c r="G13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H13" s="10">
-        <v>0.15</v>
-      </c>
-      <c r="I13" s="10">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="8">
-        <v>1</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="H14" s="12">
-        <v>1.36</v>
-      </c>
-      <c r="I14" s="10">
-        <f t="shared" si="0"/>
-        <v>1.36</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>139</v>
       </c>
       <c r="F15" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="G15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H15" s="10">
-        <v>0.86</v>
-      </c>
-      <c r="I15" s="10">
-        <f>H15*B15</f>
-        <v>0.86</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="18">
+        <v>3.49</v>
+      </c>
+      <c r="J15" s="18">
+        <f>I15*B15</f>
+        <v>3.49</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
+        <v>141</v>
+      </c>
+      <c r="D16" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" t="s">
+        <v>149</v>
+      </c>
+      <c r="F16" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" t="s">
+        <v>151</v>
+      </c>
+      <c r="H16" t="s">
+        <v>151</v>
+      </c>
+      <c r="I16" s="9">
+        <v>0.32</v>
+      </c>
+      <c r="J16" s="9">
+        <f>I16*B16</f>
+        <v>0.32</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" t="s">
+        <v>139</v>
+      </c>
+      <c r="F17" t="s">
+        <v>86</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="I17" s="9">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="J17" s="9">
+        <f>I17*B17</f>
+        <v>2.2799999999999998</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G18" t="s">
+        <v>13</v>
+      </c>
+      <c r="I18" s="9">
+        <f>12.76/10</f>
+        <v>1.276</v>
+      </c>
+      <c r="J18" s="9">
+        <f>I18*B18</f>
+        <v>2.552</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" t="s">
+        <v>140</v>
+      </c>
+      <c r="F19" t="s">
+        <v>80</v>
+      </c>
+      <c r="G19" t="s">
+        <v>81</v>
+      </c>
+      <c r="I19" s="9">
+        <v>0.73</v>
+      </c>
+      <c r="J19" s="9">
+        <f>I19*B19</f>
+        <v>0.73</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="H20" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="D16" t="s">
-        <v>90</v>
-      </c>
-      <c r="E16" t="s">
-        <v>91</v>
-      </c>
-      <c r="F16" t="s">
-        <v>92</v>
-      </c>
-      <c r="G16" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="H16" s="19">
-        <v>4.58</v>
-      </c>
-      <c r="I16" s="19">
-        <f>H16*B16</f>
-        <v>4.58</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" t="s">
-        <v>97</v>
-      </c>
-      <c r="F17" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" t="s">
-        <v>98</v>
-      </c>
-      <c r="H17" s="10">
-        <v>0.73</v>
-      </c>
-      <c r="I17" s="10">
-        <v>0.73</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s">
-        <v>100</v>
-      </c>
-      <c r="D18" t="s">
-        <v>101</v>
-      </c>
-      <c r="E18" t="s">
-        <v>102</v>
-      </c>
-      <c r="F18" t="s">
-        <v>103</v>
-      </c>
-      <c r="G18" t="s">
-        <v>103</v>
-      </c>
-      <c r="H18" s="10">
-        <v>0.14199999999999999</v>
-      </c>
-      <c r="I18" s="10">
-        <f>H18*B18</f>
-        <v>0.14199999999999999</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B19">
-        <v>2</v>
-      </c>
-      <c r="C19" t="s">
-        <v>105</v>
-      </c>
-      <c r="D19" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E19" t="s">
-        <v>107</v>
-      </c>
-      <c r="F19" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="G19" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="H19" s="15">
-        <v>1.17</v>
-      </c>
-      <c r="I19" s="10">
-        <f>H19*B19</f>
-        <v>2.34</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="G20" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="H20" s="15">
-        <f>(B2*H2)+(B3*H3)+(B4*H4)+(B5*H5)+(B6*H6)+(B7*H7)+(B8*H8)+(B9*H9)+(B10*H10)+(B11*H11)+(B12*H12)+(B13*H13)+(B14*H14)+(B15*H15)+(B16*H16)+(B17*H17)+(B18*H18)+(B19*H19)</f>
-        <v>25.971999999999998</v>
-      </c>
-      <c r="I20" s="15">
-        <f>SUM(I2:I19)</f>
-        <v>25.971999999999998</v>
-      </c>
-      <c r="K20" s="15"/>
-      <c r="L20" s="15"/>
+      <c r="I20" s="14">
+        <f>(B2*I2)+(B18*I18)+(B3*I3)+(B4*I4)+(B5*I5)+(B6*I6)+(B7*I7)+(B8*I8)+(B9*I9)+(B10*I10)+(B11*I11)+(B12*I12)+(B13*I13)+(B14*I14)+(B15*I15)+(B19*I19)+(B16*I16)+(B17*I17)</f>
+        <v>24.012000000000004</v>
+      </c>
+      <c r="J20" s="14">
+        <f>SUM(J2:J19)</f>
+        <v>24.012000000000004</v>
+      </c>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J13" r:id="rId1" xr:uid="{69F1C53A-BA78-4BEC-BCEF-44C8CF21CED4}"/>
-    <hyperlink ref="J3" r:id="rId2" xr:uid="{E8322F0E-BBAF-48E3-983F-BE52783AB5B0}"/>
-    <hyperlink ref="J6" r:id="rId3" xr:uid="{752CDDA8-D9FA-450E-967C-627E74DC45F6}"/>
-    <hyperlink ref="J4" r:id="rId4" xr:uid="{067A63A0-2652-4D61-BC70-255F0E9BEB4D}"/>
-    <hyperlink ref="J9" r:id="rId5" xr:uid="{7B637549-DF2C-434D-B6DC-2338F06F62CC}"/>
-    <hyperlink ref="J7" r:id="rId6" xr:uid="{6D4318D9-0EFC-4F26-8277-859B9AA7846C}"/>
-    <hyperlink ref="J5" r:id="rId7" xr:uid="{D79C6B18-F2C9-462E-A325-2BFBCE1FCB39}"/>
-    <hyperlink ref="J11" r:id="rId8" xr:uid="{79510C97-647E-4AC0-BAB9-4BDFD3E72D91}"/>
-    <hyperlink ref="J14" r:id="rId9" xr:uid="{C77A552B-D0A6-4664-8F30-6B5E92FDF2ED}"/>
-    <hyperlink ref="J2" r:id="rId10" xr:uid="{8EF9FDB8-6366-48C1-88DE-B9A0E3877605}"/>
-    <hyperlink ref="J18" r:id="rId11" xr:uid="{96E2D4AA-0BE4-435A-91FA-576996A3ABFE}"/>
-    <hyperlink ref="J12" r:id="rId12" xr:uid="{03D9F01E-EE38-4760-8619-2EB695295147}"/>
-    <hyperlink ref="J8" r:id="rId13" xr:uid="{47DD13C4-BBCE-4053-9D85-EF5F38771F8A}"/>
-    <hyperlink ref="J19" r:id="rId14" xr:uid="{C472B03E-D0EA-4CD5-B832-8DFF674F5416}"/>
+    <hyperlink ref="K12" r:id="rId1" xr:uid="{69F1C53A-BA78-4BEC-BCEF-44C8CF21CED4}"/>
+    <hyperlink ref="K5" r:id="rId2" xr:uid="{752CDDA8-D9FA-450E-967C-627E74DC45F6}"/>
+    <hyperlink ref="K3" r:id="rId3" xr:uid="{067A63A0-2652-4D61-BC70-255F0E9BEB4D}"/>
+    <hyperlink ref="K8" r:id="rId4" xr:uid="{7B637549-DF2C-434D-B6DC-2338F06F62CC}"/>
+    <hyperlink ref="K6" r:id="rId5" xr:uid="{6D4318D9-0EFC-4F26-8277-859B9AA7846C}"/>
+    <hyperlink ref="K10" r:id="rId6" xr:uid="{79510C97-647E-4AC0-BAB9-4BDFD3E72D91}"/>
+    <hyperlink ref="K13" r:id="rId7" xr:uid="{C77A552B-D0A6-4664-8F30-6B5E92FDF2ED}"/>
+    <hyperlink ref="K16" r:id="rId8" xr:uid="{96E2D4AA-0BE4-435A-91FA-576996A3ABFE}"/>
+    <hyperlink ref="K11" r:id="rId9" xr:uid="{03D9F01E-EE38-4760-8619-2EB695295147}"/>
+    <hyperlink ref="K7" r:id="rId10" xr:uid="{47DD13C4-BBCE-4053-9D85-EF5F38771F8A}"/>
+    <hyperlink ref="K17" r:id="rId11" xr:uid="{C472B03E-D0EA-4CD5-B832-8DFF674F5416}"/>
+    <hyperlink ref="K4" r:id="rId12" xr:uid="{CDC69774-A033-496F-9B61-40F5B5DC03CA}"/>
+    <hyperlink ref="K9" r:id="rId13" xr:uid="{85EB62F2-6BA9-4AE4-B90B-AFDA6ECEE6BB}"/>
+    <hyperlink ref="K2" r:id="rId14" xr:uid="{509E509D-C606-4116-B161-279087C0DAAE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId15"/>
@@ -1647,37 +1705,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="J1" s="13" t="s">
+      <c r="C1" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="12" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1686,37 +1744,37 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E2" s="17">
+        <v>99</v>
+      </c>
+      <c r="E2" s="16">
         <v>24.82</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="15">
         <v>2</v>
       </c>
-      <c r="G2" s="17">
+      <c r="G2" s="16">
         <v>15</v>
       </c>
-      <c r="H2" s="17">
+      <c r="H2" s="16">
         <f>E2+F2+G2</f>
         <v>41.82</v>
       </c>
-      <c r="I2" s="17">
+      <c r="I2" s="16">
         <f t="shared" ref="I2:I51" si="0">H2*1.33</f>
         <v>55.620600000000003</v>
       </c>
-      <c r="J2" s="17">
+      <c r="J2" s="16">
         <f>I2/A2</f>
         <v>11.124120000000001</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1724,37 +1782,37 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>123</v>
-      </c>
-      <c r="E3" s="17">
+        <v>101</v>
+      </c>
+      <c r="E3" s="16">
         <v>20.22</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="15">
         <v>2</v>
       </c>
-      <c r="G3" s="17">
+      <c r="G3" s="16">
         <v>15</v>
       </c>
-      <c r="H3" s="17">
+      <c r="H3" s="16">
         <f t="shared" ref="H3:H51" si="1">E3+F3+G3</f>
         <v>37.22</v>
       </c>
-      <c r="I3" s="17">
+      <c r="I3" s="16">
         <f t="shared" si="0"/>
         <v>49.502600000000001</v>
       </c>
-      <c r="J3" s="17">
+      <c r="J3" s="16">
         <f t="shared" ref="J3:J51" si="2">I3/A3</f>
         <v>9.9005200000000002</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1762,37 +1820,37 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C4" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>124</v>
-      </c>
-      <c r="E4" s="17">
+        <v>102</v>
+      </c>
+      <c r="E4" s="16">
         <v>9.4700000000000006</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="15">
         <v>2</v>
       </c>
-      <c r="G4" s="17">
+      <c r="G4" s="16">
         <v>0</v>
       </c>
-      <c r="H4" s="17">
+      <c r="H4" s="16">
         <f t="shared" si="1"/>
         <v>11.47</v>
       </c>
-      <c r="I4" s="17">
+      <c r="I4" s="16">
         <f t="shared" si="0"/>
         <v>15.255100000000002</v>
       </c>
-      <c r="J4" s="17">
+      <c r="J4" s="16">
         <f t="shared" si="2"/>
         <v>3.0510200000000003</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1800,37 +1858,37 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>121</v>
-      </c>
-      <c r="E5" s="17">
+        <v>99</v>
+      </c>
+      <c r="E5" s="16">
         <v>24.82</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="15">
         <v>5</v>
       </c>
-      <c r="G5" s="17">
+      <c r="G5" s="16">
         <v>15</v>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="16">
         <f t="shared" si="1"/>
         <v>44.82</v>
       </c>
-      <c r="I5" s="17">
+      <c r="I5" s="16">
         <f t="shared" si="0"/>
         <v>59.610600000000005</v>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="16">
         <f t="shared" si="2"/>
         <v>5.9610600000000007</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1838,37 +1896,37 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C6" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E6" s="17">
+        <v>101</v>
+      </c>
+      <c r="E6" s="16">
         <v>20.22</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="15">
         <v>5</v>
       </c>
-      <c r="G6" s="17">
+      <c r="G6" s="16">
         <v>15</v>
       </c>
-      <c r="H6" s="17">
+      <c r="H6" s="16">
         <f t="shared" si="1"/>
         <v>40.22</v>
       </c>
-      <c r="I6" s="17">
+      <c r="I6" s="16">
         <f t="shared" si="0"/>
         <v>53.492600000000003</v>
       </c>
-      <c r="J6" s="17">
+      <c r="J6" s="16">
         <f t="shared" si="2"/>
         <v>5.3492600000000001</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1876,37 +1934,37 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E7" s="17">
+        <v>102</v>
+      </c>
+      <c r="E7" s="16">
         <v>9.4700000000000006</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="15">
         <v>5</v>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="16">
         <v>0</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="16">
         <f t="shared" si="1"/>
         <v>14.47</v>
       </c>
-      <c r="I7" s="17">
+      <c r="I7" s="16">
         <f t="shared" si="0"/>
         <v>19.245100000000001</v>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="16">
         <f t="shared" si="2"/>
         <v>1.9245100000000002</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1914,37 +1972,37 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E8" s="17">
+        <v>99</v>
+      </c>
+      <c r="E8" s="16">
         <v>24.82</v>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="16">
         <v>12.8</v>
       </c>
-      <c r="G8" s="17">
+      <c r="G8" s="16">
         <v>15</v>
       </c>
-      <c r="H8" s="17">
+      <c r="H8" s="16">
         <f t="shared" si="1"/>
         <v>52.620000000000005</v>
       </c>
-      <c r="I8" s="17">
+      <c r="I8" s="16">
         <f t="shared" si="0"/>
         <v>69.984600000000015</v>
       </c>
-      <c r="J8" s="17">
+      <c r="J8" s="16">
         <f t="shared" si="2"/>
         <v>1.3996920000000004</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1952,37 +2010,37 @@
         <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C9" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
-      </c>
-      <c r="E9" s="17">
+        <v>99</v>
+      </c>
+      <c r="E9" s="16">
         <v>24.82</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="16">
         <v>27.3</v>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="16">
         <v>15</v>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="16">
         <f t="shared" si="1"/>
         <v>67.12</v>
       </c>
-      <c r="I9" s="17">
+      <c r="I9" s="16">
         <f t="shared" si="0"/>
         <v>89.269600000000011</v>
       </c>
-      <c r="J9" s="17">
+      <c r="J9" s="16">
         <f t="shared" si="2"/>
         <v>1.7853920000000003</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1990,37 +2048,37 @@
         <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C10" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>123</v>
-      </c>
-      <c r="E10" s="17">
+        <v>101</v>
+      </c>
+      <c r="E10" s="16">
         <v>20.22</v>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="16">
         <v>12.8</v>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="16">
         <v>15</v>
       </c>
-      <c r="H10" s="17">
+      <c r="H10" s="16">
         <f t="shared" si="1"/>
         <v>48.019999999999996</v>
       </c>
-      <c r="I10" s="17">
+      <c r="I10" s="16">
         <f t="shared" si="0"/>
         <v>63.866599999999998</v>
       </c>
-      <c r="J10" s="17">
+      <c r="J10" s="16">
         <f t="shared" si="2"/>
         <v>1.2773319999999999</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -2028,37 +2086,37 @@
         <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C11" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
-        <v>123</v>
-      </c>
-      <c r="E11" s="17">
+        <v>101</v>
+      </c>
+      <c r="E11" s="16">
         <v>20.22</v>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="16">
         <v>27.3</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="16">
         <v>15</v>
       </c>
-      <c r="H11" s="17">
+      <c r="H11" s="16">
         <f t="shared" si="1"/>
         <v>62.519999999999996</v>
       </c>
-      <c r="I11" s="17">
+      <c r="I11" s="16">
         <f t="shared" si="0"/>
         <v>83.151600000000002</v>
       </c>
-      <c r="J11" s="17">
+      <c r="J11" s="16">
         <f t="shared" si="2"/>
         <v>1.6630320000000001</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -2066,37 +2124,37 @@
         <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C12" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="D12" t="s">
-        <v>124</v>
-      </c>
-      <c r="E12" s="17">
+        <v>102</v>
+      </c>
+      <c r="E12" s="16">
         <v>13.29</v>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="16">
         <v>12.8</v>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="16">
         <v>0</v>
       </c>
-      <c r="H12" s="17">
+      <c r="H12" s="16">
         <f t="shared" si="1"/>
         <v>26.09</v>
       </c>
-      <c r="I12" s="17">
+      <c r="I12" s="16">
         <f t="shared" si="0"/>
         <v>34.6997</v>
       </c>
-      <c r="J12" s="17">
+      <c r="J12" s="16">
         <f t="shared" si="2"/>
         <v>0.693994</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -2104,37 +2162,37 @@
         <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C13" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="D13" t="s">
-        <v>124</v>
-      </c>
-      <c r="E13" s="17">
+        <v>102</v>
+      </c>
+      <c r="E13" s="16">
         <v>13.29</v>
       </c>
-      <c r="F13" s="17">
+      <c r="F13" s="16">
         <v>27.3</v>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="16">
         <v>0</v>
       </c>
-      <c r="H13" s="17">
+      <c r="H13" s="16">
         <f t="shared" si="1"/>
         <v>40.590000000000003</v>
       </c>
-      <c r="I13" s="17">
+      <c r="I13" s="16">
         <f t="shared" si="0"/>
         <v>53.984700000000011</v>
       </c>
-      <c r="J13" s="17">
+      <c r="J13" s="16">
         <f t="shared" si="2"/>
         <v>1.0796940000000002</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -2142,37 +2200,37 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C14" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D14" t="s">
-        <v>123</v>
-      </c>
-      <c r="E14" s="16">
+        <v>101</v>
+      </c>
+      <c r="E14" s="15">
         <v>21</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="15">
         <v>5</v>
       </c>
-      <c r="G14" s="17">
+      <c r="G14" s="16">
         <v>15</v>
       </c>
-      <c r="H14" s="17">
+      <c r="H14" s="16">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="I14" s="17">
+      <c r="I14" s="16">
         <f t="shared" si="0"/>
         <v>54.53</v>
       </c>
-      <c r="J14" s="17">
+      <c r="J14" s="16">
         <f>I14/A14</f>
         <v>10.906000000000001</v>
       </c>
       <c r="K14" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -2180,37 +2238,37 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C15" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>130</v>
-      </c>
-      <c r="E15" s="16">
+        <v>108</v>
+      </c>
+      <c r="E15" s="15">
         <v>7</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="15">
         <v>5</v>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="16">
         <v>0</v>
       </c>
-      <c r="H15" s="17">
+      <c r="H15" s="16">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I15" s="17">
+      <c r="I15" s="16">
         <f t="shared" si="0"/>
         <v>15.96</v>
       </c>
-      <c r="J15" s="17">
+      <c r="J15" s="16">
         <f t="shared" si="2"/>
         <v>3.1920000000000002</v>
       </c>
       <c r="K15" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -2218,37 +2276,37 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C16" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D16" t="s">
-        <v>131</v>
-      </c>
-      <c r="E16" s="16">
+        <v>109</v>
+      </c>
+      <c r="E16" s="15">
         <v>6</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="15">
         <v>5</v>
       </c>
-      <c r="G16" s="17">
+      <c r="G16" s="16">
         <v>0</v>
       </c>
-      <c r="H16" s="17">
+      <c r="H16" s="16">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="I16" s="17">
+      <c r="I16" s="16">
         <f t="shared" si="0"/>
         <v>14.63</v>
       </c>
-      <c r="J16" s="17">
+      <c r="J16" s="16">
         <f t="shared" si="2"/>
         <v>2.9260000000000002</v>
       </c>
       <c r="K16" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -2256,37 +2314,37 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C17" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D17" t="s">
-        <v>132</v>
-      </c>
-      <c r="E17" s="16">
+        <v>110</v>
+      </c>
+      <c r="E17" s="15">
         <v>26</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="15">
         <v>5</v>
       </c>
-      <c r="G17" s="17">
+      <c r="G17" s="16">
         <v>15</v>
       </c>
-      <c r="H17" s="17">
+      <c r="H17" s="16">
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
-      <c r="I17" s="17">
+      <c r="I17" s="16">
         <f t="shared" si="0"/>
         <v>61.180000000000007</v>
       </c>
-      <c r="J17" s="17">
+      <c r="J17" s="16">
         <f t="shared" si="2"/>
         <v>12.236000000000001</v>
       </c>
       <c r="K17" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -2294,37 +2352,37 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C18" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D18" t="s">
-        <v>123</v>
-      </c>
-      <c r="E18" s="16">
+        <v>101</v>
+      </c>
+      <c r="E18" s="15">
         <v>21</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="15">
         <v>5</v>
       </c>
-      <c r="G18" s="17">
+      <c r="G18" s="16">
         <v>15</v>
       </c>
-      <c r="H18" s="17">
+      <c r="H18" s="16">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="I18" s="17">
+      <c r="I18" s="16">
         <f t="shared" si="0"/>
         <v>54.53</v>
       </c>
-      <c r="J18" s="17">
+      <c r="J18" s="16">
         <f t="shared" si="2"/>
         <v>5.4530000000000003</v>
       </c>
       <c r="K18" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -2332,37 +2390,37 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C19" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D19" t="s">
-        <v>133</v>
-      </c>
-      <c r="E19" s="16">
+        <v>111</v>
+      </c>
+      <c r="E19" s="15">
         <v>7</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="15">
         <v>5</v>
       </c>
-      <c r="G19" s="17">
+      <c r="G19" s="16">
         <v>0</v>
       </c>
-      <c r="H19" s="17">
+      <c r="H19" s="16">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I19" s="17">
+      <c r="I19" s="16">
         <f t="shared" si="0"/>
         <v>15.96</v>
       </c>
-      <c r="J19" s="17">
+      <c r="J19" s="16">
         <f t="shared" si="2"/>
         <v>1.5960000000000001</v>
       </c>
       <c r="K19" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -2370,37 +2428,37 @@
         <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C20" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D20" t="s">
-        <v>134</v>
-      </c>
-      <c r="E20" s="16">
+        <v>112</v>
+      </c>
+      <c r="E20" s="15">
         <v>7</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="15">
         <v>5</v>
       </c>
-      <c r="G20" s="17">
+      <c r="G20" s="16">
         <v>0</v>
       </c>
-      <c r="H20" s="17">
+      <c r="H20" s="16">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I20" s="17">
+      <c r="I20" s="16">
         <f t="shared" si="0"/>
         <v>15.96</v>
       </c>
-      <c r="J20" s="17">
+      <c r="J20" s="16">
         <f t="shared" si="2"/>
         <v>1.5960000000000001</v>
       </c>
       <c r="K20" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2408,37 +2466,37 @@
         <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D21" t="s">
-        <v>132</v>
-      </c>
-      <c r="E21" s="16">
+        <v>110</v>
+      </c>
+      <c r="E21" s="15">
         <v>26</v>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="15">
         <v>5</v>
       </c>
-      <c r="G21" s="17">
+      <c r="G21" s="16">
         <v>15</v>
       </c>
-      <c r="H21" s="17">
+      <c r="H21" s="16">
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
-      <c r="I21" s="17">
+      <c r="I21" s="16">
         <f t="shared" si="0"/>
         <v>61.180000000000007</v>
       </c>
-      <c r="J21" s="17">
+      <c r="J21" s="16">
         <f t="shared" si="2"/>
         <v>6.1180000000000003</v>
       </c>
       <c r="K21" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2446,37 +2504,37 @@
         <v>50</v>
       </c>
       <c r="B22" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D22" t="s">
-        <v>123</v>
-      </c>
-      <c r="E22" s="16">
+        <v>101</v>
+      </c>
+      <c r="E22" s="15">
         <v>28</v>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="15">
         <v>27</v>
       </c>
-      <c r="G22" s="17">
+      <c r="G22" s="16">
         <v>15</v>
       </c>
-      <c r="H22" s="17">
+      <c r="H22" s="16">
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="I22" s="17">
+      <c r="I22" s="16">
         <f t="shared" si="0"/>
         <v>93.100000000000009</v>
       </c>
-      <c r="J22" s="17">
+      <c r="J22" s="16">
         <f t="shared" si="2"/>
         <v>1.8620000000000001</v>
       </c>
       <c r="K22" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2484,37 +2542,37 @@
         <v>50</v>
       </c>
       <c r="B23" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D23" t="s">
-        <v>133</v>
-      </c>
-      <c r="E23" s="16">
+        <v>111</v>
+      </c>
+      <c r="E23" s="15">
         <v>11</v>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="15">
         <v>27</v>
       </c>
-      <c r="G23" s="17">
+      <c r="G23" s="16">
         <v>0</v>
       </c>
-      <c r="H23" s="17">
+      <c r="H23" s="16">
         <f t="shared" si="1"/>
         <v>38</v>
       </c>
-      <c r="I23" s="17">
+      <c r="I23" s="16">
         <f t="shared" si="0"/>
         <v>50.540000000000006</v>
       </c>
-      <c r="J23" s="17">
+      <c r="J23" s="16">
         <f>I23/A23</f>
         <v>1.0108000000000001</v>
       </c>
       <c r="K23" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -2522,37 +2580,37 @@
         <v>50</v>
       </c>
       <c r="B24" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D24" t="s">
-        <v>134</v>
-      </c>
-      <c r="E24" s="16">
+        <v>112</v>
+      </c>
+      <c r="E24" s="15">
         <v>11</v>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="15">
         <v>27</v>
       </c>
-      <c r="G24" s="17">
+      <c r="G24" s="16">
         <v>0</v>
       </c>
-      <c r="H24" s="17">
+      <c r="H24" s="16">
         <f t="shared" si="1"/>
         <v>38</v>
       </c>
-      <c r="I24" s="17">
+      <c r="I24" s="16">
         <f t="shared" si="0"/>
         <v>50.540000000000006</v>
       </c>
-      <c r="J24" s="17">
+      <c r="J24" s="16">
         <f t="shared" si="2"/>
         <v>1.0108000000000001</v>
       </c>
       <c r="K24" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2560,37 +2618,37 @@
         <v>50</v>
       </c>
       <c r="B25" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D25" t="s">
-        <v>132</v>
-      </c>
-      <c r="E25" s="16">
+        <v>110</v>
+      </c>
+      <c r="E25" s="15">
         <v>26</v>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="15">
         <v>27</v>
       </c>
-      <c r="G25" s="17">
+      <c r="G25" s="16">
         <v>15</v>
       </c>
-      <c r="H25" s="17">
+      <c r="H25" s="16">
         <f t="shared" si="1"/>
         <v>68</v>
       </c>
-      <c r="I25" s="17">
+      <c r="I25" s="16">
         <f t="shared" si="0"/>
         <v>90.44</v>
       </c>
-      <c r="J25" s="17">
+      <c r="J25" s="16">
         <f t="shared" si="2"/>
         <v>1.8088</v>
       </c>
       <c r="K25" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -2598,37 +2656,37 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C26" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D26" t="s">
-        <v>137</v>
-      </c>
-      <c r="E26" s="16">
+        <v>115</v>
+      </c>
+      <c r="E26" s="15">
         <v>23.8</v>
       </c>
-      <c r="F26" s="16">
+      <c r="F26" s="15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="G26" s="17">
+      <c r="G26" s="16">
         <v>15</v>
       </c>
-      <c r="H26" s="17">
+      <c r="H26" s="16">
         <f t="shared" si="1"/>
         <v>43.7</v>
       </c>
-      <c r="I26" s="17">
+      <c r="I26" s="16">
         <f t="shared" si="0"/>
         <v>58.121000000000009</v>
       </c>
-      <c r="J26" s="17">
+      <c r="J26" s="16">
         <f t="shared" si="2"/>
         <v>11.624200000000002</v>
       </c>
       <c r="K26" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2636,37 +2694,37 @@
         <v>5</v>
       </c>
       <c r="B27" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C27" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D27" t="s">
-        <v>139</v>
-      </c>
-      <c r="E27" s="17">
+        <v>117</v>
+      </c>
+      <c r="E27" s="16">
         <v>24.55</v>
       </c>
-      <c r="F27" s="16">
+      <c r="F27" s="15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="G27" s="17">
+      <c r="G27" s="16">
         <v>15</v>
       </c>
-      <c r="H27" s="17">
+      <c r="H27" s="16">
         <f t="shared" si="1"/>
         <v>44.45</v>
       </c>
-      <c r="I27" s="17">
+      <c r="I27" s="16">
         <f t="shared" si="0"/>
         <v>59.118500000000004</v>
       </c>
-      <c r="J27" s="17">
+      <c r="J27" s="16">
         <f t="shared" si="2"/>
         <v>11.823700000000001</v>
       </c>
       <c r="K27" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2674,37 +2732,37 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C28" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D28" t="s">
-        <v>137</v>
-      </c>
-      <c r="E28" s="16">
+        <v>115</v>
+      </c>
+      <c r="E28" s="15">
         <v>23.8</v>
       </c>
-      <c r="F28" s="16">
+      <c r="F28" s="15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="G28" s="17">
+      <c r="G28" s="16">
         <v>15</v>
       </c>
-      <c r="H28" s="17">
+      <c r="H28" s="16">
         <f t="shared" si="1"/>
         <v>43.7</v>
       </c>
-      <c r="I28" s="17">
+      <c r="I28" s="16">
         <f t="shared" si="0"/>
         <v>58.121000000000009</v>
       </c>
-      <c r="J28" s="17">
+      <c r="J28" s="16">
         <f t="shared" si="2"/>
         <v>5.8121000000000009</v>
       </c>
       <c r="K28" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2712,37 +2770,37 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C29" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D29" t="s">
-        <v>139</v>
-      </c>
-      <c r="E29" s="17">
+        <v>117</v>
+      </c>
+      <c r="E29" s="16">
         <v>24.55</v>
       </c>
-      <c r="F29" s="16">
+      <c r="F29" s="15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="G29" s="17">
+      <c r="G29" s="16">
         <v>15</v>
       </c>
-      <c r="H29" s="17">
+      <c r="H29" s="16">
         <f t="shared" si="1"/>
         <v>44.45</v>
       </c>
-      <c r="I29" s="17">
+      <c r="I29" s="16">
         <f t="shared" si="0"/>
         <v>59.118500000000004</v>
       </c>
-      <c r="J29" s="17">
+      <c r="J29" s="16">
         <f t="shared" si="2"/>
         <v>5.9118500000000003</v>
       </c>
       <c r="K29" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2750,37 +2808,37 @@
         <v>50</v>
       </c>
       <c r="B30" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C30" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D30" t="s">
-        <v>137</v>
-      </c>
-      <c r="E30" s="17">
+        <v>115</v>
+      </c>
+      <c r="E30" s="16">
         <v>26.7</v>
       </c>
-      <c r="F30" s="17">
+      <c r="F30" s="16">
         <v>26.36</v>
       </c>
-      <c r="G30" s="17">
+      <c r="G30" s="16">
         <v>15</v>
       </c>
-      <c r="H30" s="17">
+      <c r="H30" s="16">
         <f t="shared" si="1"/>
         <v>68.06</v>
       </c>
-      <c r="I30" s="17">
+      <c r="I30" s="16">
         <f t="shared" si="0"/>
         <v>90.519800000000004</v>
       </c>
-      <c r="J30" s="17">
+      <c r="J30" s="16">
         <f t="shared" si="2"/>
         <v>1.8103960000000001</v>
       </c>
       <c r="K30" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -2788,37 +2846,37 @@
         <v>50</v>
       </c>
       <c r="B31" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D31" t="s">
-        <v>139</v>
-      </c>
-      <c r="E31" s="17">
+        <v>117</v>
+      </c>
+      <c r="E31" s="16">
         <v>28.54</v>
       </c>
-      <c r="F31" s="17">
+      <c r="F31" s="16">
         <v>26.36</v>
       </c>
-      <c r="G31" s="17">
+      <c r="G31" s="16">
         <v>15</v>
       </c>
-      <c r="H31" s="17">
+      <c r="H31" s="16">
         <f t="shared" si="1"/>
         <v>69.900000000000006</v>
       </c>
-      <c r="I31" s="17">
+      <c r="I31" s="16">
         <f t="shared" si="0"/>
         <v>92.967000000000013</v>
       </c>
-      <c r="J31" s="17">
+      <c r="J31" s="16">
         <f t="shared" si="2"/>
         <v>1.8593400000000002</v>
       </c>
       <c r="K31" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2826,37 +2884,37 @@
         <v>100</v>
       </c>
       <c r="B32" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C32" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D32" t="s">
-        <v>137</v>
-      </c>
-      <c r="E32" s="17">
+        <v>115</v>
+      </c>
+      <c r="E32" s="16">
         <v>29.6</v>
       </c>
-      <c r="F32" s="17">
+      <c r="F32" s="16">
         <v>39.130000000000003</v>
       </c>
-      <c r="G32" s="17">
+      <c r="G32" s="16">
         <v>15</v>
       </c>
-      <c r="H32" s="17">
+      <c r="H32" s="16">
         <f t="shared" si="1"/>
         <v>83.73</v>
       </c>
-      <c r="I32" s="17">
+      <c r="I32" s="16">
         <f t="shared" si="0"/>
         <v>111.36090000000002</v>
       </c>
-      <c r="J32" s="17">
+      <c r="J32" s="16">
         <f t="shared" si="2"/>
         <v>1.1136090000000001</v>
       </c>
       <c r="K32" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2864,37 +2922,37 @@
         <v>100</v>
       </c>
       <c r="B33" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="C33" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D33" t="s">
-        <v>139</v>
-      </c>
-      <c r="E33" s="17">
+        <v>117</v>
+      </c>
+      <c r="E33" s="16">
         <v>32.5</v>
       </c>
-      <c r="F33" s="17">
+      <c r="F33" s="16">
         <v>39.130000000000003</v>
       </c>
-      <c r="G33" s="17">
+      <c r="G33" s="16">
         <v>15</v>
       </c>
-      <c r="H33" s="17">
+      <c r="H33" s="16">
         <f t="shared" si="1"/>
         <v>86.63</v>
       </c>
-      <c r="I33" s="17">
+      <c r="I33" s="16">
         <f t="shared" si="0"/>
         <v>115.2179</v>
       </c>
-      <c r="J33" s="17">
+      <c r="J33" s="16">
         <f t="shared" si="2"/>
         <v>1.1521790000000001</v>
       </c>
       <c r="K33" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2902,19 +2960,19 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C34" t="s">
-        <v>141</v>
-      </c>
-      <c r="F34" s="16">
+        <v>119</v>
+      </c>
+      <c r="F34" s="15">
         <v>15.85</v>
       </c>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="16"/>
       <c r="K34" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2922,19 +2980,19 @@
         <v>6</v>
       </c>
       <c r="B35" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C35" t="s">
-        <v>141</v>
-      </c>
-      <c r="F35" s="16">
+        <v>119</v>
+      </c>
+      <c r="F35" s="15">
         <v>31.7</v>
       </c>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
       <c r="K35" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2942,19 +3000,19 @@
         <v>9</v>
       </c>
       <c r="B36" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C36" t="s">
-        <v>141</v>
-      </c>
-      <c r="F36" s="17">
+        <v>119</v>
+      </c>
+      <c r="F36" s="16">
         <v>47.55</v>
       </c>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
       <c r="K36" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2962,19 +3020,19 @@
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C37" t="s">
-        <v>141</v>
-      </c>
-      <c r="F37" s="17">
+        <v>119</v>
+      </c>
+      <c r="F37" s="16">
         <v>63.4</v>
       </c>
-      <c r="H37" s="17"/>
-      <c r="I37" s="17"/>
-      <c r="J37" s="17"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
       <c r="K37" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2982,19 +3040,19 @@
         <v>21</v>
       </c>
       <c r="B38" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C38" t="s">
-        <v>141</v>
-      </c>
-      <c r="F38" s="17">
+        <v>119</v>
+      </c>
+      <c r="F38" s="16">
         <v>110.95</v>
       </c>
-      <c r="H38" s="17"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="16"/>
       <c r="K38" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -3002,19 +3060,19 @@
         <v>51</v>
       </c>
       <c r="B39" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C39" t="s">
-        <v>141</v>
-      </c>
-      <c r="F39" s="17">
+        <v>119</v>
+      </c>
+      <c r="F39" s="16">
         <v>269.45</v>
       </c>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
-      <c r="J39" s="17"/>
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
       <c r="K39" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -3022,19 +3080,19 @@
         <v>102</v>
       </c>
       <c r="B40" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C40" t="s">
-        <v>141</v>
-      </c>
-      <c r="F40" s="17">
+        <v>119</v>
+      </c>
+      <c r="F40" s="16">
         <v>538.9</v>
       </c>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
       <c r="K40" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -3042,19 +3100,19 @@
         <v>3</v>
       </c>
       <c r="B41" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F41" s="17">
+        <v>121</v>
+      </c>
+      <c r="F41" s="16">
         <v>31.7</v>
       </c>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="17"/>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="16"/>
       <c r="K41" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -3062,19 +3120,19 @@
         <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C42" t="s">
-        <v>143</v>
-      </c>
-      <c r="F42" s="17">
+        <v>121</v>
+      </c>
+      <c r="F42" s="16">
         <v>63.4</v>
       </c>
-      <c r="H42" s="17"/>
-      <c r="I42" s="17"/>
-      <c r="J42" s="17"/>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16"/>
+      <c r="J42" s="16"/>
       <c r="K42" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -3082,19 +3140,19 @@
         <v>9</v>
       </c>
       <c r="B43" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C43" t="s">
-        <v>143</v>
-      </c>
-      <c r="F43" s="16">
+        <v>121</v>
+      </c>
+      <c r="F43" s="15">
         <v>95.1</v>
       </c>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
+      <c r="H43" s="16"/>
+      <c r="I43" s="16"/>
+      <c r="J43" s="16"/>
       <c r="K43" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -3102,19 +3160,19 @@
         <v>12</v>
       </c>
       <c r="B44" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C44" t="s">
-        <v>143</v>
-      </c>
-      <c r="F44" s="17">
+        <v>121</v>
+      </c>
+      <c r="F44" s="16">
         <v>126.8</v>
       </c>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="16"/>
       <c r="K44" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
@@ -3122,19 +3180,19 @@
         <v>21</v>
       </c>
       <c r="B45" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C45" t="s">
-        <v>143</v>
-      </c>
-      <c r="F45" s="17">
+        <v>121</v>
+      </c>
+      <c r="F45" s="16">
         <v>221.9</v>
       </c>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
+      <c r="H45" s="16"/>
+      <c r="I45" s="16"/>
+      <c r="J45" s="16"/>
       <c r="K45" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -3142,19 +3200,19 @@
         <v>51</v>
       </c>
       <c r="B46" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C46" t="s">
-        <v>143</v>
-      </c>
-      <c r="F46" s="17">
+        <v>121</v>
+      </c>
+      <c r="F46" s="16">
         <v>538.9</v>
       </c>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
+      <c r="H46" s="16"/>
+      <c r="I46" s="16"/>
+      <c r="J46" s="16"/>
       <c r="K46" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -3162,19 +3220,19 @@
         <v>102</v>
       </c>
       <c r="B47" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C47" t="s">
-        <v>143</v>
-      </c>
-      <c r="F47" s="17">
+        <v>121</v>
+      </c>
+      <c r="F47" s="16">
         <v>1077.8</v>
       </c>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="16"/>
       <c r="K47" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3182,19 +3240,19 @@
         <v>40</v>
       </c>
       <c r="B48" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C48" t="s">
-        <v>144</v>
-      </c>
-      <c r="F48" s="17">
+        <v>122</v>
+      </c>
+      <c r="F48" s="16">
         <v>126.8</v>
       </c>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17"/>
-      <c r="J48" s="17"/>
+      <c r="H48" s="16"/>
+      <c r="I48" s="16"/>
+      <c r="J48" s="16"/>
       <c r="K48" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -3202,19 +3260,19 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C49" t="s">
-        <v>144</v>
-      </c>
-      <c r="F49" s="17">
+        <v>122</v>
+      </c>
+      <c r="F49" s="16">
         <v>158.5</v>
       </c>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
+      <c r="H49" s="16"/>
+      <c r="I49" s="16"/>
+      <c r="J49" s="16"/>
       <c r="K49" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -3222,37 +3280,37 @@
         <v>100</v>
       </c>
       <c r="B50" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C50" t="s">
-        <v>144</v>
+        <v>122</v>
       </c>
       <c r="D50" t="s">
-        <v>145</v>
-      </c>
-      <c r="E50" s="16">
+        <v>123</v>
+      </c>
+      <c r="E50" s="15">
         <v>0</v>
       </c>
-      <c r="F50" s="16">
+      <c r="F50" s="15">
         <v>317</v>
       </c>
-      <c r="G50" s="16">
+      <c r="G50" s="15">
         <v>0</v>
       </c>
-      <c r="H50" s="17">
+      <c r="H50" s="16">
         <f t="shared" si="1"/>
         <v>317</v>
       </c>
-      <c r="I50" s="17">
+      <c r="I50" s="16">
         <f t="shared" si="0"/>
         <v>421.61</v>
       </c>
-      <c r="J50" s="17">
+      <c r="J50" s="16">
         <f t="shared" si="2"/>
         <v>4.2161</v>
       </c>
       <c r="K50" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -3260,32 +3318,32 @@
         <v>100</v>
       </c>
       <c r="B51" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C51" t="s">
-        <v>144</v>
+        <v>122</v>
       </c>
       <c r="D51" t="s">
-        <v>146</v>
-      </c>
-      <c r="E51" s="16">
+        <v>124</v>
+      </c>
+      <c r="E51" s="15">
         <v>33</v>
       </c>
-      <c r="F51" s="16">
+      <c r="F51" s="15">
         <v>317</v>
       </c>
-      <c r="G51" s="17">
+      <c r="G51" s="16">
         <v>15</v>
       </c>
-      <c r="H51" s="17">
+      <c r="H51" s="16">
         <f t="shared" si="1"/>
         <v>365</v>
       </c>
-      <c r="I51" s="17">
+      <c r="I51" s="16">
         <f t="shared" si="0"/>
         <v>485.45000000000005</v>
       </c>
-      <c r="J51" s="17">
+      <c r="J51" s="16">
         <f t="shared" si="2"/>
         <v>4.8545000000000007</v>
       </c>
@@ -3295,7 +3353,7 @@
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>147</v>
+        <v>125</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -3303,7 +3361,7 @@
         <v>2</v>
       </c>
       <c r="C54" t="s">
-        <v>148</v>
+        <v>126</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -3311,7 +3369,7 @@
         <v>3</v>
       </c>
       <c r="C55" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>